<commit_message>
Make a database for Imported rows
</commit_message>
<xml_diff>
--- a/sample_data/1_Standard_Format.xlsx
+++ b/sample_data/1_Standard_Format.xlsx
@@ -514,7 +514,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Grace Hardware Supply Inc.</t>
+          <t>[TEST] Grace Hardware Supply Inc.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -529,7 +529,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>201-333-444-000</t>
+          <t>999-100-100-000</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -581,7 +581,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Blessed Trading Co.</t>
+          <t>[TEST] Blessed Trading Co.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -596,7 +596,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>202-444-555-000</t>
+          <t>999-100-200-000</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -652,7 +652,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>New Life Office Supplies</t>
+          <t>[TEST] New Life Office Supplies</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -667,7 +667,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>203-555-666-000</t>
+          <t>999-100-300-000</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -715,7 +715,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Faithful Catering Services</t>
+          <t>[TEST] Faithful Catering Services</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -730,7 +730,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>204-666-777-000</t>
+          <t>999-100-400-000</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -782,7 +782,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Covenant IT Solutions</t>
+          <t>[TEST] Covenant IT Solutions</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -797,7 +797,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>205-777-888-000</t>
+          <t>999-100-500-000</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -849,7 +849,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Cornerstone Audio Visual</t>
+          <t>[TEST] Cornerstone Audio Visual</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>206-888-999-000</t>
+          <t>999-100-600-000</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">

</xml_diff>